<commit_message>
zscore fully implemented and extended to prices
</commit_message>
<xml_diff>
--- a/outputs/Beans_(fava,_dry)_percentile_classification_matrix.xlsx
+++ b/outputs/Beans_(fava,_dry)_percentile_classification_matrix.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2128" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2128" uniqueCount="106">
   <si>
     <t>2020 Mar</t>
   </si>
@@ -331,46 +331,7 @@
     <t>No data</t>
   </si>
   <si>
-    <t>Alert</t>
-  </si>
-  <si>
-    <t>Alarm</t>
-  </si>
-  <si>
     <t>0%</t>
-  </si>
-  <si>
-    <t>11%</t>
-  </si>
-  <si>
-    <t>6%</t>
-  </si>
-  <si>
-    <t>3%</t>
-  </si>
-  <si>
-    <t>14%</t>
-  </si>
-  <si>
-    <t>7%</t>
-  </si>
-  <si>
-    <t>4%</t>
-  </si>
-  <si>
-    <t>8%</t>
-  </si>
-  <si>
-    <t>1%</t>
-  </si>
-  <si>
-    <t>10%</t>
-  </si>
-  <si>
-    <t>19%</t>
-  </si>
-  <si>
-    <t>18%</t>
   </si>
 </sst>
 </file>
@@ -997,7 +958,7 @@
         <v>104</v>
       </c>
       <c r="E2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F2" t="s">
         <v>103</v>
@@ -1027,10 +988,10 @@
         <v>103</v>
       </c>
       <c r="O2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="P2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="Q2" t="s">
         <v>104</v>
@@ -1042,22 +1003,22 @@
         <v>103</v>
       </c>
       <c r="T2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="U2" t="s">
         <v>103</v>
       </c>
       <c r="V2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="W2" t="s">
         <v>104</v>
       </c>
       <c r="X2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="Y2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="Z2" t="s">
         <v>104</v>
@@ -1204,13 +1165,13 @@
         <v>104</v>
       </c>
       <c r="BV2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BW2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BX2" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:76">
@@ -1368,10 +1329,10 @@
         <v>104</v>
       </c>
       <c r="AZ3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BA3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BB3" t="s">
         <v>104</v>
@@ -1419,7 +1380,7 @@
         <v>104</v>
       </c>
       <c r="BQ3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BR3" t="s">
         <v>104</v>
@@ -1434,13 +1395,13 @@
         <v>104</v>
       </c>
       <c r="BV3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BW3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BX3" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:76">
@@ -1598,7 +1559,7 @@
         <v>103</v>
       </c>
       <c r="AZ4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BA4" t="s">
         <v>104</v>
@@ -1610,16 +1571,16 @@
         <v>103</v>
       </c>
       <c r="BD4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BE4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BF4" t="s">
         <v>104</v>
       </c>
       <c r="BG4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BH4" t="s">
         <v>104</v>
@@ -1637,19 +1598,19 @@
         <v>104</v>
       </c>
       <c r="BM4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BN4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BO4" t="s">
         <v>103</v>
       </c>
       <c r="BP4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BQ4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BR4" t="s">
         <v>104</v>
@@ -1658,19 +1619,19 @@
         <v>104</v>
       </c>
       <c r="BT4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BU4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BV4" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="BW4" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="BX4" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:76">
@@ -1840,7 +1801,7 @@
         <v>103</v>
       </c>
       <c r="BD5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BE5" t="s">
         <v>103</v>
@@ -1849,22 +1810,22 @@
         <v>103</v>
       </c>
       <c r="BG5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BH5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BI5" t="s">
         <v>103</v>
       </c>
       <c r="BJ5" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BK5" t="s">
         <v>104</v>
       </c>
       <c r="BL5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BM5" t="s">
         <v>103</v>
@@ -1876,7 +1837,7 @@
         <v>103</v>
       </c>
       <c r="BP5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BQ5" t="s">
         <v>103</v>
@@ -1885,7 +1846,7 @@
         <v>103</v>
       </c>
       <c r="BS5" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BT5" t="s">
         <v>104</v>
@@ -1894,13 +1855,13 @@
         <v>104</v>
       </c>
       <c r="BV5" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="BW5" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="BX5" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
     </row>
     <row r="6" spans="1:76">
@@ -2040,7 +2001,7 @@
         <v>103</v>
       </c>
       <c r="AT6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AU6" t="s">
         <v>104</v>
@@ -2052,10 +2013,10 @@
         <v>103</v>
       </c>
       <c r="AX6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AY6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AZ6" t="s">
         <v>103</v>
@@ -2064,28 +2025,28 @@
         <v>103</v>
       </c>
       <c r="BB6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BC6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BD6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BE6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BF6" t="s">
         <v>104</v>
       </c>
       <c r="BG6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BH6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BI6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BJ6" t="s">
         <v>104</v>
@@ -2124,13 +2085,13 @@
         <v>104</v>
       </c>
       <c r="BV6" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BW6" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
       <c r="BX6" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
     </row>
     <row r="7" spans="1:76">
@@ -2336,10 +2297,10 @@
         <v>104</v>
       </c>
       <c r="BP7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BQ7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BR7" t="s">
         <v>104</v>
@@ -2354,13 +2315,13 @@
         <v>104</v>
       </c>
       <c r="BV7" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BW7" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BX7" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="8" spans="1:76">
@@ -2437,7 +2398,7 @@
         <v>103</v>
       </c>
       <c r="Y8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="Z8" t="s">
         <v>104</v>
@@ -2452,7 +2413,7 @@
         <v>103</v>
       </c>
       <c r="AD8" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AE8" t="s">
         <v>104</v>
@@ -2533,7 +2494,7 @@
         <v>104</v>
       </c>
       <c r="BE8" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BF8" t="s">
         <v>103</v>
@@ -2584,13 +2545,13 @@
         <v>104</v>
       </c>
       <c r="BV8" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BW8" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="BX8" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
     </row>
     <row r="9" spans="1:76">
@@ -2625,16 +2586,16 @@
         <v>103</v>
       </c>
       <c r="K9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="L9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="M9" t="s">
         <v>103</v>
       </c>
       <c r="N9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O9" t="s">
         <v>103</v>
@@ -2643,7 +2604,7 @@
         <v>104</v>
       </c>
       <c r="Q9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="R9" t="s">
         <v>104</v>
@@ -2655,7 +2616,7 @@
         <v>103</v>
       </c>
       <c r="U9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="V9" t="s">
         <v>103</v>
@@ -2676,7 +2637,7 @@
         <v>103</v>
       </c>
       <c r="AB9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AC9" t="s">
         <v>104</v>
@@ -2814,13 +2775,13 @@
         <v>104</v>
       </c>
       <c r="BV9" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BW9" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BX9" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="10" spans="1:76">
@@ -2942,25 +2903,25 @@
         <v>104</v>
       </c>
       <c r="AN10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AO10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AP10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AQ10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AR10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AS10" t="s">
         <v>103</v>
       </c>
       <c r="AT10" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AU10" t="s">
         <v>104</v>
@@ -3038,19 +2999,19 @@
         <v>104</v>
       </c>
       <c r="BT10" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BU10" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BV10" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="BW10" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BX10" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
     <row r="11" spans="1:76">
@@ -3259,10 +3220,10 @@
         <v>104</v>
       </c>
       <c r="BQ11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BR11" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BS11" t="s">
         <v>104</v>
@@ -3274,13 +3235,13 @@
         <v>104</v>
       </c>
       <c r="BV11" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BW11" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BX11" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" spans="1:76">
@@ -3426,7 +3387,7 @@
         <v>104</v>
       </c>
       <c r="AV12" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AW12" t="s">
         <v>104</v>
@@ -3444,7 +3405,7 @@
         <v>104</v>
       </c>
       <c r="BB12" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BC12" t="s">
         <v>104</v>
@@ -3483,7 +3444,7 @@
         <v>104</v>
       </c>
       <c r="BO12" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BP12" t="s">
         <v>104</v>
@@ -3504,13 +3465,13 @@
         <v>104</v>
       </c>
       <c r="BV12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BW12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BX12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:76">
@@ -3668,61 +3629,61 @@
         <v>103</v>
       </c>
       <c r="AZ13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BA13" t="s">
         <v>104</v>
       </c>
       <c r="BB13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BC13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BD13" t="s">
         <v>104</v>
       </c>
       <c r="BE13" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BF13" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BG13" t="s">
         <v>104</v>
       </c>
       <c r="BH13" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BI13" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BJ13" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BK13" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BL13" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BM13" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BN13" t="s">
         <v>104</v>
       </c>
       <c r="BO13" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BP13" t="s">
         <v>104</v>
       </c>
       <c r="BQ13" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BR13" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BS13" t="s">
         <v>103</v>
@@ -3734,13 +3695,13 @@
         <v>104</v>
       </c>
       <c r="BV13" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="BW13" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="BX13" t="s">
-        <v>117</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:76">
@@ -3895,7 +3856,7 @@
         <v>103</v>
       </c>
       <c r="AY14" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="AZ14" t="s">
         <v>103</v>
@@ -3904,13 +3865,13 @@
         <v>103</v>
       </c>
       <c r="BB14" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BC14" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BD14" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BE14" t="s">
         <v>103</v>
@@ -3922,7 +3883,7 @@
         <v>104</v>
       </c>
       <c r="BH14" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BI14" t="s">
         <v>103</v>
@@ -3931,46 +3892,46 @@
         <v>103</v>
       </c>
       <c r="BK14" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BL14" t="s">
         <v>103</v>
       </c>
       <c r="BM14" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BN14" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BO14" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BP14" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BQ14" t="s">
         <v>103</v>
       </c>
       <c r="BR14" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BS14" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BT14" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BU14" t="s">
         <v>103</v>
       </c>
       <c r="BV14" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="BW14" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="BX14" t="s">
-        <v>118</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:76">
@@ -4002,7 +3963,7 @@
         <v>104</v>
       </c>
       <c r="J15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="K15" t="s">
         <v>103</v>
@@ -4086,7 +4047,7 @@
         <v>103</v>
       </c>
       <c r="AL15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AM15" t="s">
         <v>104</v>
@@ -4119,7 +4080,7 @@
         <v>104</v>
       </c>
       <c r="AW15" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="AX15" t="s">
         <v>104</v>
@@ -4179,7 +4140,7 @@
         <v>103</v>
       </c>
       <c r="BQ15" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BR15" t="s">
         <v>104</v>
@@ -4194,13 +4155,13 @@
         <v>104</v>
       </c>
       <c r="BV15" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BW15" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="BX15" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16" spans="1:76">
@@ -4217,10 +4178,10 @@
         <v>103</v>
       </c>
       <c r="E16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="G16" t="s">
         <v>104</v>
@@ -4370,16 +4331,16 @@
         <v>103</v>
       </c>
       <c r="BD16" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BE16" t="s">
         <v>103</v>
       </c>
       <c r="BF16" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BG16" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BH16" t="s">
         <v>104</v>
@@ -4391,10 +4352,10 @@
         <v>104</v>
       </c>
       <c r="BK16" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BL16" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BM16" t="s">
         <v>104</v>
@@ -4403,7 +4364,7 @@
         <v>104</v>
       </c>
       <c r="BO16" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BP16" t="s">
         <v>104</v>
@@ -4415,7 +4376,7 @@
         <v>104</v>
       </c>
       <c r="BS16" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BT16" t="s">
         <v>104</v>
@@ -4424,13 +4385,13 @@
         <v>104</v>
       </c>
       <c r="BV16" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="BW16" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="BX16" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
     </row>
     <row r="17" spans="1:76">
@@ -4606,10 +4567,10 @@
         <v>103</v>
       </c>
       <c r="BF17" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BG17" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BH17" t="s">
         <v>104</v>
@@ -4618,16 +4579,16 @@
         <v>103</v>
       </c>
       <c r="BJ17" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BK17" t="s">
         <v>104</v>
       </c>
       <c r="BL17" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BM17" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BN17" t="s">
         <v>104</v>
@@ -4645,7 +4606,7 @@
         <v>104</v>
       </c>
       <c r="BS17" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BT17" t="s">
         <v>103</v>
@@ -4654,13 +4615,13 @@
         <v>104</v>
       </c>
       <c r="BV17" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="BW17" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="BX17" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
     </row>
     <row r="18" spans="1:76">
@@ -4728,7 +4689,7 @@
         <v>104</v>
       </c>
       <c r="V18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="W18" t="s">
         <v>103</v>
@@ -4743,7 +4704,7 @@
         <v>103</v>
       </c>
       <c r="AA18" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AB18" t="s">
         <v>103</v>
@@ -4830,7 +4791,7 @@
         <v>104</v>
       </c>
       <c r="BD18" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BE18" t="s">
         <v>104</v>
@@ -4884,13 +4845,13 @@
         <v>104</v>
       </c>
       <c r="BV18" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BW18" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="BX18" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
     </row>
     <row r="19" spans="1:76">
@@ -5075,22 +5036,22 @@
         <v>104</v>
       </c>
       <c r="BI19" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BJ19" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BK19" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BL19" t="s">
         <v>103</v>
       </c>
       <c r="BM19" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BN19" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BO19" t="s">
         <v>103</v>
@@ -5114,13 +5075,13 @@
         <v>104</v>
       </c>
       <c r="BV19" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="BW19" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="BX19" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
     </row>
     <row r="20" spans="1:76">
@@ -5266,13 +5227,13 @@
         <v>104</v>
       </c>
       <c r="AV20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AW20" t="s">
         <v>103</v>
       </c>
       <c r="AX20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AY20" t="s">
         <v>104</v>
@@ -5287,19 +5248,19 @@
         <v>104</v>
       </c>
       <c r="BC20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BD20" t="s">
         <v>104</v>
       </c>
       <c r="BE20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BF20" t="s">
         <v>103</v>
       </c>
       <c r="BG20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BH20" t="s">
         <v>104</v>
@@ -5317,7 +5278,7 @@
         <v>103</v>
       </c>
       <c r="BM20" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BN20" t="s">
         <v>104</v>
@@ -5344,13 +5305,13 @@
         <v>104</v>
       </c>
       <c r="BV20" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BW20" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BX20" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" spans="1:76">
@@ -5460,7 +5421,7 @@
         <v>103</v>
       </c>
       <c r="AJ21" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AK21" t="s">
         <v>103</v>
@@ -5544,13 +5505,13 @@
         <v>104</v>
       </c>
       <c r="BL21" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BM21" t="s">
         <v>104</v>
       </c>
       <c r="BN21" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BO21" t="s">
         <v>103</v>
@@ -5562,7 +5523,7 @@
         <v>103</v>
       </c>
       <c r="BR21" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BS21" t="s">
         <v>104</v>
@@ -5574,13 +5535,13 @@
         <v>104</v>
       </c>
       <c r="BV21" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="BW21" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BX21" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
     </row>
     <row r="22" spans="1:76">
@@ -5744,13 +5705,13 @@
         <v>104</v>
       </c>
       <c r="BB22" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BC22" t="s">
         <v>104</v>
       </c>
       <c r="BD22" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BE22" t="s">
         <v>104</v>
@@ -5765,19 +5726,19 @@
         <v>103</v>
       </c>
       <c r="BI22" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BJ22" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BK22" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BL22" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BM22" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BN22" t="s">
         <v>104</v>
@@ -5786,13 +5747,13 @@
         <v>104</v>
       </c>
       <c r="BP22" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BQ22" t="s">
         <v>103</v>
       </c>
       <c r="BR22" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BS22" t="s">
         <v>103</v>
@@ -5801,16 +5762,16 @@
         <v>103</v>
       </c>
       <c r="BU22" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BV22" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="BW22" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="BX22" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
     </row>
     <row r="23" spans="1:76">
@@ -5875,7 +5836,7 @@
         <v>103</v>
       </c>
       <c r="U23" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="V23" t="s">
         <v>104</v>
@@ -5890,7 +5851,7 @@
         <v>103</v>
       </c>
       <c r="Z23" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AA23" t="s">
         <v>104</v>
@@ -5986,7 +5947,7 @@
         <v>104</v>
       </c>
       <c r="BF23" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BG23" t="s">
         <v>104</v>
@@ -6007,10 +5968,10 @@
         <v>104</v>
       </c>
       <c r="BM23" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BN23" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BO23" t="s">
         <v>104</v>
@@ -6028,19 +5989,19 @@
         <v>103</v>
       </c>
       <c r="BT23" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BU23" t="s">
         <v>104</v>
       </c>
       <c r="BV23" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BW23" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="BX23" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
     </row>
     <row r="24" spans="1:76">
@@ -6198,7 +6159,7 @@
         <v>103</v>
       </c>
       <c r="AZ24" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BA24" t="s">
         <v>103</v>
@@ -6225,7 +6186,7 @@
         <v>104</v>
       </c>
       <c r="BI24" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BJ24" t="s">
         <v>104</v>
@@ -6243,7 +6204,7 @@
         <v>103</v>
       </c>
       <c r="BO24" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BP24" t="s">
         <v>103</v>
@@ -6255,7 +6216,7 @@
         <v>103</v>
       </c>
       <c r="BS24" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BT24" t="s">
         <v>104</v>
@@ -6264,13 +6225,13 @@
         <v>104</v>
       </c>
       <c r="BV24" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BW24" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BX24" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="25" spans="1:76">
@@ -6410,10 +6371,10 @@
         <v>104</v>
       </c>
       <c r="AT25" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AU25" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AV25" t="s">
         <v>103</v>
@@ -6461,7 +6422,7 @@
         <v>103</v>
       </c>
       <c r="BK25" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BL25" t="s">
         <v>104</v>
@@ -6473,7 +6434,7 @@
         <v>103</v>
       </c>
       <c r="BO25" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BP25" t="s">
         <v>104</v>
@@ -6494,13 +6455,13 @@
         <v>104</v>
       </c>
       <c r="BV25" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BW25" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="BX25" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="26" spans="1:76">
@@ -6688,13 +6649,13 @@
         <v>104</v>
       </c>
       <c r="BJ26" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BK26" t="s">
         <v>103</v>
       </c>
       <c r="BL26" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BM26" t="s">
         <v>103</v>
@@ -6703,7 +6664,7 @@
         <v>103</v>
       </c>
       <c r="BO26" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BP26" t="s">
         <v>103</v>
@@ -6712,7 +6673,7 @@
         <v>103</v>
       </c>
       <c r="BR26" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="BS26" t="s">
         <v>104</v>
@@ -6724,13 +6685,13 @@
         <v>104</v>
       </c>
       <c r="BV26" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="BW26" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="BX26" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
     </row>
     <row r="27" spans="1:76">
@@ -6900,7 +6861,7 @@
         <v>104</v>
       </c>
       <c r="BD27" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="BE27" t="s">
         <v>104</v>
@@ -6912,7 +6873,7 @@
         <v>104</v>
       </c>
       <c r="BH27" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BI27" t="s">
         <v>103</v>
@@ -6921,7 +6882,7 @@
         <v>103</v>
       </c>
       <c r="BK27" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BL27" t="s">
         <v>103</v>
@@ -6939,7 +6900,7 @@
         <v>104</v>
       </c>
       <c r="BQ27" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BR27" t="s">
         <v>103</v>
@@ -6954,13 +6915,13 @@
         <v>104</v>
       </c>
       <c r="BV27" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
       <c r="BW27" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="BX27" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
     </row>
     <row r="28" spans="1:76">
@@ -7067,7 +7028,7 @@
         <v>103</v>
       </c>
       <c r="AI28" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="AJ28" t="s">
         <v>103</v>
@@ -7079,7 +7040,7 @@
         <v>103</v>
       </c>
       <c r="AM28" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="AN28" t="s">
         <v>104</v>
@@ -7154,16 +7115,16 @@
         <v>104</v>
       </c>
       <c r="BL28" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BM28" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BN28" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BO28" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BP28" t="s">
         <v>104</v>
@@ -7178,19 +7139,19 @@
         <v>104</v>
       </c>
       <c r="BT28" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BU28" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="BV28" t="s">
-        <v>114</v>
+        <v>105</v>
       </c>
       <c r="BW28" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="BX28" t="s">
-        <v>116</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>